<commit_message>
Add Implemenation for wavelet and mean removel preprocessing approaches
</commit_message>
<xml_diff>
--- a/Task 1_EOG Task/matrix_features.xlsx
+++ b/Task 1_EOG Task/matrix_features.xlsx
@@ -463,25 +463,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>-2.853585284177109e-17</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>3.020666325532341</v>
+        <v>3.184269880285294</v>
       </c>
       <c r="E2" t="n">
-        <v>189.591993355157</v>
+        <v>154.6738465902048</v>
       </c>
       <c r="F2" t="n">
-        <v>2.808756045035638</v>
+        <v>2.674755283254382</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.722227985100539</v>
+        <v>-2.50995396705369</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9123750034848005</v>
+        <v>0.8318801603503666</v>
       </c>
     </row>
     <row r="3">
@@ -489,25 +489,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>2.486899575160351e-17</v>
+        <v>1.426792642088554e-17</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>3.319088526439866</v>
+        <v>2.917190321425021</v>
       </c>
       <c r="E3" t="n">
-        <v>142.7131581202464</v>
+        <v>182.3660832475351</v>
       </c>
       <c r="F3" t="n">
-        <v>2.805815080165402</v>
+        <v>2.586078685359078</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.714107379441963</v>
+        <v>-2.396191865600748</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9067779409417626</v>
+        <v>0.8041287905695562</v>
       </c>
     </row>
     <row r="4">
@@ -515,25 +515,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>5.684341886080802e-17</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>1.330348770790658</v>
+        <v>2.66361473151912</v>
       </c>
       <c r="E4" t="n">
-        <v>224.4078365013508</v>
+        <v>187.9322079364477</v>
       </c>
       <c r="F4" t="n">
-        <v>2.809262654440048</v>
+        <v>2.618957773322362</v>
       </c>
       <c r="G4" t="n">
-        <v>-2.717111658250565</v>
+        <v>-2.410673877029641</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9073186583929731</v>
+        <v>0.789725254380891</v>
       </c>
     </row>
     <row r="5">
@@ -541,25 +541,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>-1.776356839400251e-17</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>2.382042338865378</v>
+        <v>3.006318071970923</v>
       </c>
       <c r="E5" t="n">
-        <v>183.6961092757188</v>
+        <v>161.8508219821481</v>
       </c>
       <c r="F5" t="n">
-        <v>2.802987633940389</v>
+        <v>2.687696081870039</v>
       </c>
       <c r="G5" t="n">
-        <v>-2.725054515628631</v>
+        <v>-2.534013932030773</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9214856000412008</v>
+        <v>0.8442775007738573</v>
       </c>
     </row>
     <row r="6">
@@ -567,25 +567,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>-1.4210854715202e-17</v>
+        <v>2.853585284177109e-17</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>3.06137044102004</v>
+        <v>4.081793719534556</v>
       </c>
       <c r="E6" t="n">
-        <v>183.675735995431</v>
+        <v>159.6566482035748</v>
       </c>
       <c r="F6" t="n">
-        <v>2.784640541420767</v>
+        <v>2.607340026933318</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.691603344545809</v>
+        <v>-2.406368641733699</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9056908689508002</v>
+        <v>0.792737975513114</v>
       </c>
     </row>
     <row r="7">
@@ -593,25 +593,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>5.684341886080802e-17</v>
+        <v>-1.426792642088554e-17</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1.071346229604981</v>
+        <v>2.529573995798684</v>
       </c>
       <c r="E7" t="n">
-        <v>164.8142780319049</v>
+        <v>158.50917901114</v>
       </c>
       <c r="F7" t="n">
-        <v>2.801216863282584</v>
+        <v>2.638653778072024</v>
       </c>
       <c r="G7" t="n">
-        <v>-2.716473493023726</v>
+        <v>-2.442618308397357</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9138633325119543</v>
+        <v>0.7977841593063755</v>
       </c>
     </row>
     <row r="8">
@@ -619,25 +619,25 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>-8.526512829121202e-17</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>1.222591025508774</v>
+        <v>0.9192037572506113</v>
       </c>
       <c r="E8" t="n">
-        <v>154.1511749409032</v>
+        <v>130.3635499015001</v>
       </c>
       <c r="F8" t="n">
-        <v>2.820703686259905</v>
+        <v>2.643623146495946</v>
       </c>
       <c r="G8" t="n">
-        <v>-2.741041288339993</v>
+        <v>-2.460512481959873</v>
       </c>
       <c r="H8" t="n">
-        <v>0.918954469046762</v>
+        <v>0.8124039075038691</v>
       </c>
     </row>
     <row r="9">
@@ -645,25 +645,25 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>2.853585284177109e-17</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>1.030152106403006</v>
+        <v>0.9519118056267167</v>
       </c>
       <c r="E9" t="n">
-        <v>156.3008842981922</v>
+        <v>127.2098317569194</v>
       </c>
       <c r="F9" t="n">
-        <v>2.808625740469816</v>
+        <v>2.65313748345474</v>
       </c>
       <c r="G9" t="n">
-        <v>-2.72441509899379</v>
+        <v>-2.494282076924633</v>
       </c>
       <c r="H9" t="n">
-        <v>0.9140712473691228</v>
+        <v>0.835077017479777</v>
       </c>
     </row>
     <row r="10">
@@ -671,25 +671,25 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>1.4210854715202e-17</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>1.047879296838459</v>
+        <v>1.561379841378364</v>
       </c>
       <c r="E10" t="n">
-        <v>153.1754283606799</v>
+        <v>139.5682034279348</v>
       </c>
       <c r="F10" t="n">
-        <v>2.806003983590967</v>
+        <v>2.598743215852388</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.725445619872731</v>
+        <v>-2.38672314063654</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9180674445138294</v>
+        <v>0.7811959916176585</v>
       </c>
     </row>
     <row r="11">
@@ -697,25 +697,25 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>-1.13686837721616e-16</v>
+        <v>-2.853585284177109e-17</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9214685234996357</v>
+        <v>2.104740033027116</v>
       </c>
       <c r="E11" t="n">
-        <v>146.5246025242406</v>
+        <v>136.7397777899966</v>
       </c>
       <c r="F11" t="n">
-        <v>2.796233390980795</v>
+        <v>2.60554864367004</v>
       </c>
       <c r="G11" t="n">
-        <v>-2.707712486641418</v>
+        <v>-2.402909195892266</v>
       </c>
       <c r="H11" t="n">
-        <v>0.909545956707669</v>
+        <v>0.7895188604755166</v>
       </c>
     </row>
     <row r="12">
@@ -723,25 +723,25 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>5.684341886080802e-17</v>
+        <v>-2.853585284177109e-17</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>1.739532853382453</v>
+        <v>2.086129966629065</v>
       </c>
       <c r="E12" t="n">
-        <v>231.3837730836695</v>
+        <v>200.450732676</v>
       </c>
       <c r="F12" t="n">
-        <v>2.698776371804481</v>
+        <v>2.340518316059403</v>
       </c>
       <c r="G12" t="n">
-        <v>-2.635636062845604</v>
+        <v>-2.222665894039466</v>
       </c>
       <c r="H12" t="n">
-        <v>0.93634153257871</v>
+        <v>0.8717678195386874</v>
       </c>
     </row>
     <row r="13">
@@ -749,25 +749,25 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>-8.526512829121202e-17</v>
+        <v>-2.853585284177109e-17</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>1.976950089599507</v>
+        <v>2.282442363580881</v>
       </c>
       <c r="E13" t="n">
-        <v>203.1039615380869</v>
+        <v>193.0553720767754</v>
       </c>
       <c r="F13" t="n">
-        <v>2.694661223210649</v>
+        <v>2.357210137307504</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.6340339695369</v>
+        <v>-2.189093069482744</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9378587660493982</v>
+        <v>0.8208678669740223</v>
       </c>
     </row>
     <row r="14">
@@ -775,25 +775,25 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>-1.13686837721616e-16</v>
+        <v>-2.853585284177109e-17</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>1.641152095138265</v>
+        <v>3.03980526321621</v>
       </c>
       <c r="E14" t="n">
-        <v>220.213739038764</v>
+        <v>177.7915681248244</v>
       </c>
       <c r="F14" t="n">
-        <v>2.774006666063239</v>
+        <v>2.371507591208574</v>
       </c>
       <c r="G14" t="n">
-        <v>-2.708613083999024</v>
+        <v>-2.246434360919385</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9339909128647708</v>
+        <v>0.8567254833651793</v>
       </c>
     </row>
     <row r="15">
@@ -801,25 +801,25 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>-8.526512829121202e-17</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>2.43529920869506</v>
+        <v>1.855276137899434</v>
       </c>
       <c r="E15" t="n">
-        <v>197.4116601391659</v>
+        <v>186.4645126658981</v>
       </c>
       <c r="F15" t="n">
-        <v>2.726566747970378</v>
+        <v>2.479365236897915</v>
       </c>
       <c r="G15" t="n">
-        <v>-2.667529311852156</v>
+        <v>-2.37473457647457</v>
       </c>
       <c r="H15" t="n">
-        <v>0.9397013444032258</v>
+        <v>0.8891086366441734</v>
       </c>
     </row>
     <row r="16">
@@ -827,25 +827,25 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>-1.426792642088554e-17</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1.912750422390422</v>
+        <v>2.617065620589383</v>
       </c>
       <c r="E16" t="n">
-        <v>219.029071565582</v>
+        <v>183.7793567368524</v>
       </c>
       <c r="F16" t="n">
-        <v>2.706813358561929</v>
+        <v>2.418325556323287</v>
       </c>
       <c r="G16" t="n">
-        <v>-2.641343405824343</v>
+        <v>-2.270362339219805</v>
       </c>
       <c r="H16" t="n">
-        <v>0.933143106539043</v>
+        <v>0.8374456591724648</v>
       </c>
     </row>
     <row r="17">
@@ -856,22 +856,22 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>1.565905073451257</v>
+        <v>2.735614136970801</v>
       </c>
       <c r="E17" t="n">
-        <v>187.8382423192216</v>
+        <v>192.9091561625129</v>
       </c>
       <c r="F17" t="n">
-        <v>2.757230149766715</v>
+        <v>2.456899511541464</v>
       </c>
       <c r="G17" t="n">
-        <v>-2.684144410039835</v>
+        <v>-2.320488294660625</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9259538275087167</v>
+        <v>0.8571681032099141</v>
       </c>
     </row>
     <row r="18">
@@ -879,25 +879,25 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>3.197442310920451e-17</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>1.236734113459322</v>
+        <v>1.244587832259397</v>
       </c>
       <c r="E18" t="n">
-        <v>180.7727465657444</v>
+        <v>170.4691503829181</v>
       </c>
       <c r="F18" t="n">
-        <v>2.795876776805475</v>
+        <v>2.558440056315226</v>
       </c>
       <c r="G18" t="n">
-        <v>-2.701713089803179</v>
+        <v>-2.39433100004773</v>
       </c>
       <c r="H18" t="n">
-        <v>0.9048028230557231</v>
+        <v>0.8303034982997768</v>
       </c>
     </row>
     <row r="19">
@@ -905,25 +905,25 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>-7.105427357601002e-18</v>
+        <v>5.707170568354218e-17</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>1.692352905454115</v>
+        <v>1.862085236179728</v>
       </c>
       <c r="E19" t="n">
-        <v>174.504751528255</v>
+        <v>187.2766165134972</v>
       </c>
       <c r="F19" t="n">
-        <v>2.756338600597155</v>
+        <v>2.394512566956709</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.674173452194038</v>
+        <v>-2.209546283549369</v>
       </c>
       <c r="H19" t="n">
-        <v>0.9168408646696695</v>
+        <v>0.8103253411999227</v>
       </c>
     </row>
     <row r="20">
@@ -931,25 +931,25 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>-7.105427357601002e-18</v>
+        <v>2.853585284177109e-17</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>1.454331158725708</v>
+        <v>1.151054828198274</v>
       </c>
       <c r="E20" t="n">
-        <v>189.3662801204126</v>
+        <v>170.8897085539424</v>
       </c>
       <c r="F20" t="n">
-        <v>2.745656420082029</v>
+        <v>2.456534226860803</v>
       </c>
       <c r="G20" t="n">
-        <v>-2.673489938560082</v>
+        <v>-2.264093952714938</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9268300683743937</v>
+        <v>0.8039792004957873</v>
       </c>
     </row>
     <row r="21">
@@ -957,25 +957,25 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>-2.842170943040401e-17</v>
+        <v>1.426792642088554e-17</v>
       </c>
       <c r="C21" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>1.4106401895168</v>
+        <v>2.160919503775979</v>
       </c>
       <c r="E21" t="n">
-        <v>199.9384202580486</v>
+        <v>202.5136794043501</v>
       </c>
       <c r="F21" t="n">
-        <v>2.763751130976224</v>
+        <v>2.407431930957323</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.710345437651329</v>
+        <v>-2.236350017349647</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9459254969093391</v>
+        <v>0.8201006505931695</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjust Lags to 2 to make AR to B, W_1 and W_2
</commit_message>
<xml_diff>
--- a/Task 1_EOG Task/matrix_features.xlsx
+++ b/Task 1_EOG Task/matrix_features.xlsx
@@ -444,17 +444,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>AR_1</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>AR_2</t>
+          <t>W_1</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>AR_3</t>
+          <t>W_2</t>
         </is>
       </c>
     </row>
@@ -477,13 +477,13 @@
         <v>1882.700905010351</v>
       </c>
       <c r="F2" t="n">
-        <v>2.664162631073365</v>
+        <v>0.004484603540785118</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.493799883952773</v>
+        <v>1.897556868049858</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8264429182147796</v>
+        <v>-0.9164671540726764</v>
       </c>
     </row>
     <row r="3">
@@ -505,13 +505,13 @@
         <v>1808.691950697549</v>
       </c>
       <c r="F3" t="n">
-        <v>2.594993708000254</v>
+        <v>-0.004053178226709137</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.378820519748677</v>
+        <v>1.882821197701642</v>
       </c>
       <c r="H3" t="n">
-        <v>0.779799453716592</v>
+        <v>-0.9016028813252009</v>
       </c>
     </row>
     <row r="4">
@@ -533,13 +533,13 @@
         <v>2092.793399405043</v>
       </c>
       <c r="F4" t="n">
-        <v>2.617910600629939</v>
+        <v>0.0002187719174106288</v>
       </c>
       <c r="G4" t="n">
-        <v>-2.41648929012645</v>
+        <v>1.895559868942922</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7966705354951622</v>
+        <v>-0.9046984279495274</v>
       </c>
     </row>
     <row r="5">
@@ -561,13 +561,13 @@
         <v>3027.323509872382</v>
       </c>
       <c r="F5" t="n">
-        <v>2.670582249869812</v>
+        <v>0.01038729250130252</v>
       </c>
       <c r="G5" t="n">
-        <v>-2.506304648338619</v>
+        <v>1.890894480426679</v>
       </c>
       <c r="H5" t="n">
-        <v>0.834207104752587</v>
+        <v>-0.9013226120796278</v>
       </c>
     </row>
     <row r="6">
@@ -589,13 +589,13 @@
         <v>1397.619446648867</v>
       </c>
       <c r="F6" t="n">
-        <v>2.637951773038012</v>
+        <v>0.005933785232315758</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.454532926125459</v>
+        <v>1.893968303241951</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8128041140375244</v>
+        <v>-0.9141869491366852</v>
       </c>
     </row>
     <row r="7">
@@ -617,13 +617,13 @@
         <v>1829.595765041358</v>
       </c>
       <c r="F7" t="n">
-        <v>2.672047332022698</v>
+        <v>-0.01131900301768243</v>
       </c>
       <c r="G7" t="n">
-        <v>-2.505080152789988</v>
+        <v>1.901985341809378</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8293604381747751</v>
+        <v>-0.9240062336823923</v>
       </c>
     </row>
     <row r="8">
@@ -645,13 +645,13 @@
         <v>1702.303642343285</v>
       </c>
       <c r="F8" t="n">
-        <v>2.625632361529405</v>
+        <v>-0.008377461886310505</v>
       </c>
       <c r="G8" t="n">
-        <v>-2.427167268825755</v>
+        <v>1.886660539946444</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7972951239650803</v>
+        <v>-0.9080247103752912</v>
       </c>
     </row>
     <row r="9">
@@ -673,13 +673,13 @@
         <v>1666.78862015863</v>
       </c>
       <c r="F9" t="n">
-        <v>2.641268624739464</v>
+        <v>-0.005123616429699917</v>
       </c>
       <c r="G9" t="n">
-        <v>-2.4727375556341</v>
+        <v>1.88093626058108</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8270111625872189</v>
+        <v>-0.9059062345746199</v>
       </c>
     </row>
     <row r="10">
@@ -701,13 +701,13 @@
         <v>1238.189909987479</v>
       </c>
       <c r="F10" t="n">
-        <v>2.592568194958134</v>
+        <v>-0.008201750813313433</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.374117933930977</v>
+        <v>1.877829380266726</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7757489276256624</v>
+        <v>-0.9033614210233258</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1333.582411194846</v>
       </c>
       <c r="F11" t="n">
-        <v>2.61381109335534</v>
+        <v>-0.0007572027016395809</v>
       </c>
       <c r="G11" t="n">
-        <v>-2.416807677088687</v>
+        <v>1.885121158774477</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7971364898374718</v>
+        <v>-0.9141621461561609</v>
       </c>
     </row>
     <row r="12">
@@ -757,13 +757,13 @@
         <v>661.0485427656062</v>
       </c>
       <c r="F12" t="n">
-        <v>2.291888684329439</v>
+        <v>0.007694907627168857</v>
       </c>
       <c r="G12" t="n">
-        <v>-2.081306920605602</v>
+        <v>1.62943074783419</v>
       </c>
       <c r="H12" t="n">
-        <v>0.785406196648798</v>
+        <v>-0.6610875684717687</v>
       </c>
     </row>
     <row r="13">
@@ -785,13 +785,13 @@
         <v>749.1079299199494</v>
       </c>
       <c r="F13" t="n">
-        <v>2.362624516880566</v>
+        <v>0.01754600624799723</v>
       </c>
       <c r="G13" t="n">
-        <v>-2.184097966522772</v>
+        <v>1.667267342615423</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8173898022410495</v>
+        <v>-0.7037863051150252</v>
       </c>
     </row>
     <row r="14">
@@ -813,13 +813,13 @@
         <v>391.6395383573973</v>
       </c>
       <c r="F14" t="n">
-        <v>2.374733825043716</v>
+        <v>0.02019439682675769</v>
       </c>
       <c r="G14" t="n">
-        <v>-2.258408362308218</v>
+        <v>1.724447150152107</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8712000584442016</v>
+        <v>-0.8042016740541446</v>
       </c>
     </row>
     <row r="15">
@@ -841,13 +841,13 @@
         <v>683.3794892257185</v>
       </c>
       <c r="F15" t="n">
-        <v>2.468348135397913</v>
+        <v>-0.003024142503105769</v>
       </c>
       <c r="G15" t="n">
-        <v>-2.346199497829685</v>
+        <v>1.755842102977655</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8717126460757005</v>
+        <v>-0.7994380915301862</v>
       </c>
     </row>
     <row r="16">
@@ -869,13 +869,13 @@
         <v>489.3216770392081</v>
       </c>
       <c r="F16" t="n">
-        <v>2.430425667531795</v>
+        <v>0.002314749724672763</v>
       </c>
       <c r="G16" t="n">
-        <v>-2.292798839909699</v>
+        <v>1.741392153976023</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8509016361320082</v>
+        <v>-0.8171364739395859</v>
       </c>
     </row>
     <row r="17">
@@ -897,13 +897,13 @@
         <v>1081.239938432955</v>
       </c>
       <c r="F17" t="n">
-        <v>2.443231127272561</v>
+        <v>-0.007466173171382062</v>
       </c>
       <c r="G17" t="n">
-        <v>-2.254365530235144</v>
+        <v>1.752424587640761</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8079581630503647</v>
+        <v>-0.772463840707349</v>
       </c>
     </row>
     <row r="18">
@@ -925,13 +925,13 @@
         <v>1023.014367090146</v>
       </c>
       <c r="F18" t="n">
-        <v>2.588428531157782</v>
+        <v>0.01971876750245083</v>
       </c>
       <c r="G18" t="n">
-        <v>-2.445462794695587</v>
+        <v>1.897677145889086</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8522502608305832</v>
+        <v>-0.9186720618304762</v>
       </c>
     </row>
     <row r="19">
@@ -953,13 +953,13 @@
         <v>699.1235936063077</v>
       </c>
       <c r="F19" t="n">
-        <v>2.395567870418104</v>
+        <v>-0.005483365084608638</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.204854515161245</v>
+        <v>1.726424357436716</v>
       </c>
       <c r="H19" t="n">
-        <v>0.804879309803432</v>
+        <v>-0.7509213437650755</v>
       </c>
     </row>
     <row r="20">
@@ -981,13 +981,13 @@
         <v>879.4674764862409</v>
       </c>
       <c r="F20" t="n">
-        <v>2.501480208449922</v>
+        <v>-0.0028698292820673</v>
       </c>
       <c r="G20" t="n">
-        <v>-2.349622124526467</v>
+        <v>1.812527351785071</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8445952242282314</v>
+        <v>-0.8322646952086501</v>
       </c>
     </row>
     <row r="21">
@@ -1009,13 +1009,13 @@
         <v>736.4648919920758</v>
       </c>
       <c r="F21" t="n">
-        <v>2.425914071653969</v>
+        <v>-0.00270002779478279</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.262926207258732</v>
+        <v>1.766210563639106</v>
       </c>
       <c r="H21" t="n">
-        <v>0.8330038345694933</v>
+        <v>-0.7904645670044605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Task 2 Files
</commit_message>
<xml_diff>
--- a/Task 1_EOG Task/matrix_features.xlsx
+++ b/Task 1_EOG Task/matrix_features.xlsx
@@ -465,25 +465,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.04193867983481732</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>12.62481688303298</v>
+        <v>14.96442976069828</v>
       </c>
       <c r="D2" t="n">
-        <v>42.55049890995906</v>
+        <v>45.01629964047864</v>
       </c>
       <c r="E2" t="n">
-        <v>1882.700905010351</v>
+        <v>2836.839058277732</v>
       </c>
       <c r="F2" t="n">
-        <v>0.004484603540785118</v>
+        <v>-0.004491942422039432</v>
       </c>
       <c r="G2" t="n">
-        <v>1.897556868049858</v>
+        <v>1.898596155209141</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.9164671540726764</v>
+        <v>-0.9125457069071463</v>
       </c>
     </row>
     <row r="3">
@@ -493,25 +493,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.6631671834762277</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>11.31829821599121</v>
+        <v>11.31923755246431</v>
       </c>
       <c r="D3" t="n">
-        <v>37.86194936925472</v>
+        <v>38.40512724882693</v>
       </c>
       <c r="E3" t="n">
-        <v>1808.691950697549</v>
+        <v>1631.010714376879</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.004053178226709137</v>
+        <v>0.001634684137302895</v>
       </c>
       <c r="G3" t="n">
-        <v>1.882821197701642</v>
+        <v>1.86631771665505</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.9016028813252009</v>
+        <v>-0.8860434107879424</v>
       </c>
     </row>
     <row r="4">
@@ -521,25 +521,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5966943950905877</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>11.4097423933942</v>
+        <v>22.28602634359307</v>
       </c>
       <c r="D4" t="n">
-        <v>29.57546438563019</v>
+        <v>29.82270818966899</v>
       </c>
       <c r="E4" t="n">
-        <v>2092.793399405043</v>
+        <v>4991.127673837686</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0002187719174106288</v>
+        <v>-0.02744503192212618</v>
       </c>
       <c r="G4" t="n">
-        <v>1.895559868942922</v>
+        <v>1.738471963755757</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.9046984279495274</v>
+        <v>-0.7452421706736181</v>
       </c>
     </row>
     <row r="5">
@@ -549,25 +549,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-1.071836361760394</v>
+        <v>-1.307398633798584e-15</v>
       </c>
       <c r="C5" t="n">
-        <v>15.84154670226093</v>
+        <v>18.44177939262827</v>
       </c>
       <c r="D5" t="n">
-        <v>42.31646569295219</v>
+        <v>43.5061852023133</v>
       </c>
       <c r="E5" t="n">
-        <v>3027.323509872382</v>
+        <v>3391.35419642043</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01038729250130252</v>
+        <v>0.003168691351359235</v>
       </c>
       <c r="G5" t="n">
-        <v>1.890894480426679</v>
+        <v>1.908524634856426</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.9013226120796278</v>
+        <v>-0.9164142680868932</v>
       </c>
     </row>
     <row r="6">
@@ -577,25 +577,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.125656685789889</v>
+        <v>2.273736754432321e-16</v>
       </c>
       <c r="C6" t="n">
-        <v>9.340039106479724</v>
+        <v>10.86860914490815</v>
       </c>
       <c r="D6" t="n">
-        <v>32.92905047183481</v>
+        <v>32.51349917361794</v>
       </c>
       <c r="E6" t="n">
-        <v>1397.619446648867</v>
+        <v>1998.97016065947</v>
       </c>
       <c r="F6" t="n">
-        <v>0.005933785232315758</v>
+        <v>-0.0003922540299901127</v>
       </c>
       <c r="G6" t="n">
-        <v>1.893968303241951</v>
+        <v>1.883307378951967</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.9141869491366852</v>
+        <v>-0.8989533575208632</v>
       </c>
     </row>
     <row r="7">
@@ -605,25 +605,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02121803948407478</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>12.37295710992074</v>
+        <v>13.89037914358618</v>
       </c>
       <c r="D7" t="n">
-        <v>13.75072142957631</v>
+        <v>15.52467548694331</v>
       </c>
       <c r="E7" t="n">
-        <v>1829.595765041358</v>
+        <v>2289.787901853451</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.01131900301768243</v>
+        <v>0.0006313852315965275</v>
       </c>
       <c r="G7" t="n">
-        <v>1.901985341809378</v>
+        <v>1.902497933176459</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.9240062336823923</v>
+        <v>-0.9202076625173833</v>
       </c>
     </row>
     <row r="8">
@@ -633,25 +633,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.052699202805373</v>
+        <v>4.547473508864641e-16</v>
       </c>
       <c r="C8" t="n">
-        <v>11.38333722585093</v>
+        <v>11.90416453343676</v>
       </c>
       <c r="D8" t="n">
-        <v>11.54784754605816</v>
+        <v>16.62916837067397</v>
       </c>
       <c r="E8" t="n">
-        <v>1702.303642343285</v>
+        <v>1834.865839889504</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.008377461886310505</v>
+        <v>-0.004338233458896515</v>
       </c>
       <c r="G8" t="n">
-        <v>1.886660539946444</v>
+        <v>1.889111138501441</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.9080247103752912</v>
+        <v>-0.9092981462712242</v>
       </c>
     </row>
     <row r="9">
@@ -661,25 +661,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.529519401738712</v>
+        <v>-6.821210263296962e-16</v>
       </c>
       <c r="C9" t="n">
-        <v>10.57953006672444</v>
+        <v>10.67270222423882</v>
       </c>
       <c r="D9" t="n">
-        <v>10.83936345630942</v>
+        <v>11.23927659288291</v>
       </c>
       <c r="E9" t="n">
-        <v>1666.78862015863</v>
+        <v>1671.72575679628</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.005123616429699917</v>
+        <v>-0.008235876689718702</v>
       </c>
       <c r="G9" t="n">
-        <v>1.88093626058108</v>
+        <v>1.883436640070564</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.9059062345746199</v>
+        <v>-0.9072710640109809</v>
       </c>
     </row>
     <row r="10">
@@ -689,25 +689,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.496373174289432</v>
+        <v>-3.410605131648481e-16</v>
       </c>
       <c r="C10" t="n">
-        <v>10.04690423934426</v>
+        <v>11.83333550665115</v>
       </c>
       <c r="D10" t="n">
-        <v>8.37809609854181</v>
+        <v>12.55382411161376</v>
       </c>
       <c r="E10" t="n">
-        <v>1238.189909987479</v>
+        <v>1812.854612877153</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.008201750813313433</v>
+        <v>0.001112394038898443</v>
       </c>
       <c r="G10" t="n">
-        <v>1.877829380266726</v>
+        <v>1.863795006967585</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.9033614210233258</v>
+        <v>-0.8837965733075137</v>
       </c>
     </row>
     <row r="11">
@@ -717,25 +717,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.3276255774014185</v>
+        <v>-4.547473508864641e-16</v>
       </c>
       <c r="C11" t="n">
-        <v>10.09989266382646</v>
+        <v>11.19129033466683</v>
       </c>
       <c r="D11" t="n">
-        <v>10.2757054683176</v>
+        <v>11.36002444162584</v>
       </c>
       <c r="E11" t="n">
-        <v>1333.582411194846</v>
+        <v>1641.443246672044</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.0007572027016395809</v>
+        <v>0.001740651330353128</v>
       </c>
       <c r="G11" t="n">
-        <v>1.885121158774477</v>
+        <v>1.876962461348259</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.9141621461561609</v>
+        <v>-0.9017132167187217</v>
       </c>
     </row>
     <row r="12">
@@ -745,25 +745,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.7217294057751567</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>3.141762626113167</v>
+        <v>6.265196992016908</v>
       </c>
       <c r="D12" t="n">
-        <v>6.626204820050633</v>
+        <v>11.48986005117166</v>
       </c>
       <c r="E12" t="n">
-        <v>661.0485427656062</v>
+        <v>1449.024786463934</v>
       </c>
       <c r="F12" t="n">
-        <v>0.007694907627168857</v>
+        <v>-0.0179950805204716</v>
       </c>
       <c r="G12" t="n">
-        <v>1.62943074783419</v>
+        <v>1.637241751672108</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.6610875684717687</v>
+        <v>-0.6509865241529407</v>
       </c>
     </row>
     <row r="13">
@@ -773,25 +773,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.973717930678466</v>
+        <v>2.273736754432321e-16</v>
       </c>
       <c r="C13" t="n">
-        <v>3.361875252422548</v>
+        <v>3.912847930310472</v>
       </c>
       <c r="D13" t="n">
-        <v>7.405222214155041</v>
+        <v>7.753484485642475</v>
       </c>
       <c r="E13" t="n">
-        <v>749.1079299199494</v>
+        <v>793.4578052541502</v>
       </c>
       <c r="F13" t="n">
-        <v>0.01754600624799723</v>
+        <v>0.006275438955393061</v>
       </c>
       <c r="G13" t="n">
-        <v>1.667267342615423</v>
+        <v>1.669822150459558</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.7037863051150252</v>
+        <v>-0.7128392645675991</v>
       </c>
     </row>
     <row r="14">
@@ -801,25 +801,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.09317679134420001</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>2.165481805600502</v>
+        <v>5.060683212556007</v>
       </c>
       <c r="D14" t="n">
-        <v>4.226239572108719</v>
+        <v>8.841940972986093</v>
       </c>
       <c r="E14" t="n">
-        <v>391.6395383573973</v>
+        <v>1112.573179800567</v>
       </c>
       <c r="F14" t="n">
-        <v>0.02019439682675769</v>
+        <v>0.01444515668982849</v>
       </c>
       <c r="G14" t="n">
-        <v>1.724447150152107</v>
+        <v>1.637477496270741</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.8042016740541446</v>
+        <v>-0.6598677682786289</v>
       </c>
     </row>
     <row r="15">
@@ -829,25 +829,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.4628749389466786</v>
+        <v>-1.13686837721616e-16</v>
       </c>
       <c r="C15" t="n">
-        <v>3.404450502870687</v>
+        <v>3.714084259652449</v>
       </c>
       <c r="D15" t="n">
-        <v>6.528910768152376</v>
+        <v>8.570389690264298</v>
       </c>
       <c r="E15" t="n">
-        <v>683.3794892257185</v>
+        <v>736.0860565501557</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.003024142503105769</v>
+        <v>-0.002768583728718031</v>
       </c>
       <c r="G15" t="n">
-        <v>1.755842102977655</v>
+        <v>1.757617475699359</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.7994380915301862</v>
+        <v>-0.7941428370831507</v>
       </c>
     </row>
     <row r="16">
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.04164407190888204</v>
+        <v>2.273736754432321e-16</v>
       </c>
       <c r="C16" t="n">
-        <v>2.470927621799356</v>
+        <v>4.741386393467464</v>
       </c>
       <c r="D16" t="n">
-        <v>5.351381895780446</v>
+        <v>9.45398885739248</v>
       </c>
       <c r="E16" t="n">
-        <v>489.3216770392081</v>
+        <v>1037.795843907584</v>
       </c>
       <c r="F16" t="n">
-        <v>0.002314749724672763</v>
+        <v>0.01011288062593115</v>
       </c>
       <c r="G16" t="n">
-        <v>1.741392153976023</v>
+        <v>1.705659600061351</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.8171364739395859</v>
+        <v>-0.7379971865572015</v>
       </c>
     </row>
     <row r="17">
@@ -885,25 +885,25 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.8534537536961482</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>5.696087032029583</v>
+        <v>5.682967076873788</v>
       </c>
       <c r="D17" t="n">
-        <v>8.690492980339789</v>
+        <v>9.084323195223476</v>
       </c>
       <c r="E17" t="n">
-        <v>1081.239938432955</v>
+        <v>1076.5849713802</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.007466173171382062</v>
+        <v>-0.003491283556131875</v>
       </c>
       <c r="G17" t="n">
-        <v>1.752424587640761</v>
+        <v>1.77939307469274</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.772463840707349</v>
+        <v>-0.8002205239389031</v>
       </c>
     </row>
     <row r="18">
@@ -913,25 +913,25 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.2388363775303455</v>
+        <v>2.842170943040401e-16</v>
       </c>
       <c r="C18" t="n">
-        <v>5.905936242638894</v>
+        <v>6.388931416768371</v>
       </c>
       <c r="D18" t="n">
-        <v>6.267387457325773</v>
+        <v>8.508099545539778</v>
       </c>
       <c r="E18" t="n">
-        <v>1023.014367090146</v>
+        <v>1152.020683733459</v>
       </c>
       <c r="F18" t="n">
-        <v>0.01971876750245083</v>
+        <v>0.005568413163281455</v>
       </c>
       <c r="G18" t="n">
-        <v>1.897677145889086</v>
+        <v>1.836575814785124</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.9186720618304762</v>
+        <v>-0.8516884700474768</v>
       </c>
     </row>
     <row r="19">
@@ -941,25 +941,25 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.4088619427754118</v>
+        <v>2.700062395888381e-16</v>
       </c>
       <c r="C19" t="n">
-        <v>4.024547954213569</v>
+        <v>4.424952291285082</v>
       </c>
       <c r="D19" t="n">
-        <v>4.87852865899832</v>
+        <v>7.657573718920148</v>
       </c>
       <c r="E19" t="n">
-        <v>699.1235936063077</v>
+        <v>789.0691624460445</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.005483365084608638</v>
+        <v>0.004577264283565593</v>
       </c>
       <c r="G19" t="n">
-        <v>1.726424357436716</v>
+        <v>1.71445592102119</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.7509213437650755</v>
+        <v>-0.7387417974849454</v>
       </c>
     </row>
     <row r="20">
@@ -969,25 +969,25 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.02100545695856192</v>
+        <v>5.684341886080802e-17</v>
       </c>
       <c r="C20" t="n">
-        <v>4.973815690164174</v>
+        <v>5.592472995963216</v>
       </c>
       <c r="D20" t="n">
-        <v>5.940702492047411</v>
+        <v>8.743832695373436</v>
       </c>
       <c r="E20" t="n">
-        <v>879.4674764862409</v>
+        <v>1061.792445706777</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0028698292820673</v>
+        <v>0.004991464861846238</v>
       </c>
       <c r="G20" t="n">
-        <v>1.812527351785071</v>
+        <v>1.755639383706688</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.8322646952086501</v>
+        <v>-0.7751220915010135</v>
       </c>
     </row>
     <row r="21">
@@ -997,25 +997,25 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.06359212389529827</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>3.998622902167345</v>
+        <v>4.499978040247661</v>
       </c>
       <c r="D21" t="n">
-        <v>5.282440815722751</v>
+        <v>7.413076702386532</v>
       </c>
       <c r="E21" t="n">
-        <v>736.4648919920758</v>
+        <v>901.4158692578281</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.00270002779478279</v>
+        <v>-0.001741258842561546</v>
       </c>
       <c r="G21" t="n">
-        <v>1.766210563639106</v>
+        <v>1.737385973654064</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.7904645670044605</v>
+        <v>-0.759946966077778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>